<commit_message>
upd: Cambios en PP
</commit_message>
<xml_diff>
--- a/public/archivos/formatoReporteNominaCalentador.xlsx
+++ b/public/archivos/formatoReporteNominaCalentador.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10811"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="11027"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/diegolopez/Documents/GitProyect/vales/apivales/public/archivos/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A043F19C-D7F3-A244-A7CB-D39A88937E39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C6C5FD9-7620-2F46-8A7A-BDED999D1A47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -210,7 +210,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -246,11 +246,104 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -266,9 +359,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -295,6 +385,39 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -318,23 +441,23 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>163284</xdr:colOff>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>269875</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>2268</xdr:rowOff>
+      <xdr:rowOff>79375</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>86177</xdr:colOff>
-      <xdr:row>9</xdr:row>
-      <xdr:rowOff>67582</xdr:rowOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>1143001</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>74549</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Imagen 1">
+        <xdr:cNvPr id="3" name="Gráfico 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C0576C21-D12C-487E-FD66-836235D61F3E}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1635D0C6-ACBC-5B48-A7E5-FBF5EDB6F1D4}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -345,25 +468,23 @@
       <xdr:blipFill>
         <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
           <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            <a:ext uri="{96DAC541-7B7A-43D3-8B79-37D633B846F1}">
+              <asvg:svgBlip xmlns:asvg="http://schemas.microsoft.com/office/drawing/2016/SVG/main" r:embed="rId2"/>
             </a:ext>
           </a:extLst>
         </a:blip>
-        <a:srcRect/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </xdr:blipFill>
-      <xdr:spPr bwMode="auto">
+      <xdr:spPr>
         <a:xfrm>
-          <a:off x="163284" y="2268"/>
-          <a:ext cx="5526768" cy="1779814"/>
+          <a:off x="936625" y="79375"/>
+          <a:ext cx="4365626" cy="1519174"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
-        <a:noFill/>
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
@@ -657,249 +778,249 @@
     <col min="17" max="17" width="12.1640625" style="4" customWidth="1"/>
     <col min="18" max="19" width="31.83203125" style="5" customWidth="1"/>
     <col min="20" max="20" width="29.5" style="5" customWidth="1"/>
-    <col min="21" max="21" width="18.83203125" style="6" customWidth="1"/>
-    <col min="22" max="22" width="18.33203125" style="6" customWidth="1"/>
-    <col min="23" max="23" width="15.33203125" style="7" customWidth="1"/>
-    <col min="24" max="24" width="16.33203125" style="7" customWidth="1"/>
-    <col min="25" max="25" width="40.6640625" style="7" customWidth="1"/>
-    <col min="26" max="26" width="30.6640625" style="7" customWidth="1"/>
-    <col min="27" max="27" width="15.83203125" style="7" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="34.1640625" style="7" customWidth="1"/>
-    <col min="29" max="29" width="16.5" style="7" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="35" style="7" customWidth="1"/>
-    <col min="31" max="16384" width="11.5" style="7"/>
+    <col min="21" max="21" width="18.83203125" style="27" customWidth="1"/>
+    <col min="22" max="22" width="18.33203125" style="27" customWidth="1"/>
+    <col min="23" max="23" width="15.33203125" style="6" customWidth="1"/>
+    <col min="24" max="24" width="16.33203125" style="6" customWidth="1"/>
+    <col min="25" max="25" width="40.6640625" style="6" customWidth="1"/>
+    <col min="26" max="26" width="30.6640625" style="6" customWidth="1"/>
+    <col min="27" max="27" width="15.83203125" style="6" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="34.1640625" style="6" customWidth="1"/>
+    <col min="29" max="29" width="16.5" style="6" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="35" style="6" customWidth="1"/>
+    <col min="31" max="16384" width="11.5" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" s="12" customFormat="1" ht="15" x14ac:dyDescent="0.2">
-      <c r="A1" s="9"/>
-      <c r="B1" s="9"/>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
-      <c r="E1" s="9"/>
-      <c r="F1" s="9"/>
-      <c r="G1" s="10"/>
-      <c r="H1" s="10"/>
-      <c r="I1" s="10"/>
-      <c r="J1" s="9"/>
-      <c r="K1" s="9"/>
-      <c r="L1" s="9"/>
-      <c r="M1" s="10"/>
-      <c r="N1" s="10"/>
-      <c r="O1" s="10"/>
-      <c r="P1" s="10"/>
-      <c r="Q1" s="9"/>
-      <c r="R1" s="10"/>
-      <c r="S1" s="10"/>
-      <c r="T1" s="10"/>
-      <c r="U1" s="11"/>
-      <c r="V1" s="11"/>
-    </row>
-    <row r="2" spans="1:35" s="12" customFormat="1" ht="15" x14ac:dyDescent="0.2">
-      <c r="A2" s="17"/>
-      <c r="B2" s="17"/>
-      <c r="C2" s="17"/>
-      <c r="D2" s="17"/>
-      <c r="E2" s="17"/>
-      <c r="F2" s="17"/>
-      <c r="G2" s="17"/>
-      <c r="H2" s="17"/>
-      <c r="I2" s="17"/>
-      <c r="J2" s="17"/>
-      <c r="K2" s="17"/>
-      <c r="L2" s="17"/>
-      <c r="M2" s="17"/>
-      <c r="N2" s="17"/>
-      <c r="O2" s="17"/>
-      <c r="P2" s="17"/>
-      <c r="Q2" s="17"/>
-      <c r="R2" s="17"/>
-      <c r="S2" s="17"/>
-      <c r="T2" s="17"/>
-      <c r="U2" s="17"/>
-      <c r="V2" s="17"/>
-    </row>
-    <row r="3" spans="1:35" s="12" customFormat="1" ht="15" x14ac:dyDescent="0.2">
-      <c r="A3" s="17"/>
-      <c r="B3" s="17"/>
-      <c r="C3" s="17"/>
-      <c r="D3" s="17"/>
-      <c r="E3" s="17"/>
-      <c r="F3" s="17"/>
-      <c r="G3" s="17"/>
-      <c r="H3" s="17"/>
-      <c r="I3" s="17"/>
-      <c r="J3" s="17"/>
-      <c r="K3" s="17"/>
-      <c r="L3" s="17"/>
-      <c r="M3" s="17"/>
-      <c r="N3" s="17"/>
-      <c r="O3" s="17"/>
-      <c r="P3" s="17"/>
-      <c r="Q3" s="17"/>
-      <c r="R3" s="17"/>
-      <c r="S3" s="17"/>
-      <c r="T3" s="17"/>
-      <c r="U3" s="17"/>
-      <c r="V3" s="17"/>
-    </row>
-    <row r="4" spans="1:35" s="12" customFormat="1" ht="15" x14ac:dyDescent="0.2">
-      <c r="A4" s="9"/>
-      <c r="B4" s="9"/>
-      <c r="C4" s="9"/>
-      <c r="D4" s="9"/>
-      <c r="E4" s="9"/>
-      <c r="F4" s="9"/>
-      <c r="G4" s="10"/>
-      <c r="H4" s="10"/>
-      <c r="I4" s="10"/>
-      <c r="J4" s="9"/>
-      <c r="K4" s="9"/>
-      <c r="L4" s="9"/>
-      <c r="M4" s="10"/>
-      <c r="N4" s="13"/>
-      <c r="O4" s="13"/>
-      <c r="P4" s="13"/>
-      <c r="Q4" s="14"/>
-      <c r="R4" s="13"/>
-      <c r="S4" s="13"/>
-      <c r="T4" s="13"/>
-      <c r="U4" s="11"/>
-      <c r="V4" s="11"/>
-    </row>
-    <row r="5" spans="1:35" s="12" customFormat="1" ht="15" x14ac:dyDescent="0.2">
-      <c r="A5" s="9"/>
-      <c r="B5" s="9"/>
-      <c r="C5" s="9"/>
-      <c r="D5" s="9"/>
-      <c r="E5" s="9"/>
-      <c r="F5" s="9"/>
-      <c r="G5" s="10"/>
-      <c r="H5" s="10"/>
-      <c r="I5" s="10"/>
-      <c r="J5" s="9"/>
-      <c r="K5" s="9"/>
-      <c r="L5" s="9"/>
-      <c r="M5" s="15"/>
-      <c r="N5" s="10"/>
-      <c r="O5" s="10"/>
-      <c r="P5" s="10"/>
-      <c r="Q5" s="9"/>
-      <c r="R5" s="10"/>
-      <c r="S5" s="10"/>
-      <c r="T5" s="10"/>
-      <c r="U5" s="11"/>
-      <c r="V5" s="11"/>
-    </row>
-    <row r="6" spans="1:35" s="12" customFormat="1" ht="15" x14ac:dyDescent="0.2">
-      <c r="A6" s="9"/>
-      <c r="B6" s="9"/>
-      <c r="C6" s="9"/>
-      <c r="D6" s="9"/>
-      <c r="E6" s="9"/>
-      <c r="F6" s="9"/>
-      <c r="G6" s="10"/>
-      <c r="H6" s="10"/>
-      <c r="I6" s="10"/>
-      <c r="J6" s="9"/>
-      <c r="K6" s="9"/>
-      <c r="L6" s="9"/>
-      <c r="M6" s="16"/>
-      <c r="N6" s="10"/>
-      <c r="O6" s="10"/>
-      <c r="P6" s="10"/>
-      <c r="Q6" s="9"/>
-      <c r="R6" s="10"/>
-      <c r="S6" s="10"/>
-      <c r="T6" s="10"/>
-      <c r="U6" s="11"/>
-      <c r="V6" s="11"/>
-    </row>
-    <row r="7" spans="1:35" s="12" customFormat="1" ht="15" x14ac:dyDescent="0.2">
-      <c r="A7" s="9"/>
-      <c r="B7" s="9"/>
-      <c r="C7" s="9"/>
-      <c r="D7" s="9"/>
-      <c r="E7" s="9"/>
-      <c r="F7" s="9"/>
-      <c r="G7" s="10"/>
-      <c r="H7" s="10"/>
-      <c r="I7" s="10"/>
-      <c r="J7" s="9"/>
-      <c r="K7" s="9"/>
-      <c r="L7" s="9"/>
-      <c r="M7" s="13"/>
-      <c r="N7" s="10"/>
-      <c r="O7" s="10"/>
-      <c r="P7" s="10"/>
-      <c r="Q7" s="9"/>
-      <c r="R7" s="10"/>
-      <c r="S7" s="10"/>
-      <c r="T7" s="10"/>
-      <c r="U7" s="11"/>
-      <c r="V7" s="11"/>
-    </row>
-    <row r="8" spans="1:35" s="12" customFormat="1" ht="15" x14ac:dyDescent="0.2">
-      <c r="A8" s="9"/>
-      <c r="B8" s="9"/>
-      <c r="C8" s="9"/>
-      <c r="D8" s="9"/>
-      <c r="E8" s="9"/>
-      <c r="F8" s="9"/>
-      <c r="G8" s="10"/>
-      <c r="H8" s="10"/>
-      <c r="I8" s="10"/>
-      <c r="J8" s="9"/>
-      <c r="K8" s="9"/>
-      <c r="L8" s="9"/>
-      <c r="M8" s="10"/>
-      <c r="N8" s="10"/>
-      <c r="O8" s="10"/>
-      <c r="P8" s="10"/>
-      <c r="Q8" s="9"/>
-      <c r="R8" s="10"/>
-      <c r="S8" s="10"/>
-      <c r="T8" s="10"/>
-      <c r="U8" s="11"/>
-      <c r="V8" s="11"/>
-    </row>
-    <row r="9" spans="1:35" s="12" customFormat="1" ht="15" x14ac:dyDescent="0.2">
-      <c r="A9" s="9"/>
-      <c r="B9" s="9"/>
-      <c r="C9" s="9"/>
-      <c r="D9" s="9"/>
-      <c r="E9" s="9"/>
-      <c r="F9" s="9"/>
-      <c r="G9" s="10"/>
-      <c r="H9" s="10"/>
-      <c r="I9" s="10"/>
-      <c r="J9" s="9"/>
-      <c r="K9" s="9"/>
-      <c r="L9" s="9"/>
-      <c r="M9" s="10"/>
-      <c r="N9" s="10"/>
-      <c r="O9" s="10"/>
-      <c r="P9" s="10"/>
-      <c r="Q9" s="9"/>
-      <c r="R9" s="10"/>
-      <c r="S9" s="10"/>
-      <c r="T9" s="10"/>
-      <c r="U9" s="11"/>
-      <c r="V9" s="11"/>
+    <row r="1" spans="1:35" s="11" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+      <c r="A1" s="8"/>
+      <c r="B1" s="18"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="20"/>
+      <c r="F1" s="8"/>
+      <c r="G1" s="9"/>
+      <c r="H1" s="9"/>
+      <c r="I1" s="9"/>
+      <c r="J1" s="8"/>
+      <c r="K1" s="8"/>
+      <c r="L1" s="8"/>
+      <c r="M1" s="9"/>
+      <c r="N1" s="9"/>
+      <c r="O1" s="9"/>
+      <c r="P1" s="9"/>
+      <c r="Q1" s="8"/>
+      <c r="R1" s="9"/>
+      <c r="S1" s="9"/>
+      <c r="T1" s="9"/>
+      <c r="U1" s="10"/>
+      <c r="V1" s="10"/>
+    </row>
+    <row r="2" spans="1:35" s="11" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+      <c r="A2" s="16"/>
+      <c r="B2" s="21"/>
+      <c r="C2" s="22"/>
+      <c r="D2" s="22"/>
+      <c r="E2" s="23"/>
+      <c r="F2" s="16"/>
+      <c r="G2" s="16"/>
+      <c r="H2" s="16"/>
+      <c r="I2" s="16"/>
+      <c r="J2" s="16"/>
+      <c r="K2" s="16"/>
+      <c r="L2" s="16"/>
+      <c r="M2" s="16"/>
+      <c r="N2" s="16"/>
+      <c r="O2" s="16"/>
+      <c r="P2" s="16"/>
+      <c r="Q2" s="16"/>
+      <c r="R2" s="16"/>
+      <c r="S2" s="16"/>
+      <c r="T2" s="16"/>
+      <c r="U2" s="16"/>
+      <c r="V2" s="16"/>
+    </row>
+    <row r="3" spans="1:35" s="11" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+      <c r="A3" s="16"/>
+      <c r="B3" s="21"/>
+      <c r="C3" s="22"/>
+      <c r="D3" s="22"/>
+      <c r="E3" s="23"/>
+      <c r="F3" s="16"/>
+      <c r="G3" s="16"/>
+      <c r="H3" s="16"/>
+      <c r="I3" s="16"/>
+      <c r="J3" s="16"/>
+      <c r="K3" s="16"/>
+      <c r="L3" s="16"/>
+      <c r="M3" s="16"/>
+      <c r="N3" s="16"/>
+      <c r="O3" s="16"/>
+      <c r="P3" s="16"/>
+      <c r="Q3" s="16"/>
+      <c r="R3" s="16"/>
+      <c r="S3" s="16"/>
+      <c r="T3" s="16"/>
+      <c r="U3" s="16"/>
+      <c r="V3" s="16"/>
+    </row>
+    <row r="4" spans="1:35" s="11" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+      <c r="A4" s="8"/>
+      <c r="B4" s="21"/>
+      <c r="C4" s="22"/>
+      <c r="D4" s="22"/>
+      <c r="E4" s="23"/>
+      <c r="F4" s="8"/>
+      <c r="G4" s="9"/>
+      <c r="H4" s="9"/>
+      <c r="I4" s="9"/>
+      <c r="J4" s="8"/>
+      <c r="K4" s="8"/>
+      <c r="L4" s="8"/>
+      <c r="M4" s="9"/>
+      <c r="N4" s="12"/>
+      <c r="O4" s="12"/>
+      <c r="P4" s="12"/>
+      <c r="Q4" s="13"/>
+      <c r="R4" s="12"/>
+      <c r="S4" s="12"/>
+      <c r="T4" s="12"/>
+      <c r="U4" s="10"/>
+      <c r="V4" s="10"/>
+    </row>
+    <row r="5" spans="1:35" s="11" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+      <c r="A5" s="8"/>
+      <c r="B5" s="21"/>
+      <c r="C5" s="22"/>
+      <c r="D5" s="22"/>
+      <c r="E5" s="23"/>
+      <c r="F5" s="8"/>
+      <c r="G5" s="9"/>
+      <c r="H5" s="9"/>
+      <c r="I5" s="9"/>
+      <c r="J5" s="8"/>
+      <c r="K5" s="8"/>
+      <c r="L5" s="8"/>
+      <c r="M5" s="14"/>
+      <c r="N5" s="9"/>
+      <c r="O5" s="9"/>
+      <c r="P5" s="9"/>
+      <c r="Q5" s="8"/>
+      <c r="R5" s="9"/>
+      <c r="S5" s="9"/>
+      <c r="T5" s="9"/>
+      <c r="U5" s="10"/>
+      <c r="V5" s="10"/>
+    </row>
+    <row r="6" spans="1:35" s="11" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+      <c r="A6" s="8"/>
+      <c r="B6" s="21"/>
+      <c r="C6" s="22"/>
+      <c r="D6" s="22"/>
+      <c r="E6" s="23"/>
+      <c r="F6" s="8"/>
+      <c r="G6" s="9"/>
+      <c r="H6" s="9"/>
+      <c r="I6" s="9"/>
+      <c r="J6" s="8"/>
+      <c r="K6" s="8"/>
+      <c r="L6" s="8"/>
+      <c r="M6" s="15"/>
+      <c r="N6" s="9"/>
+      <c r="O6" s="9"/>
+      <c r="P6" s="9"/>
+      <c r="Q6" s="8"/>
+      <c r="R6" s="9"/>
+      <c r="S6" s="9"/>
+      <c r="T6" s="9"/>
+      <c r="U6" s="10"/>
+      <c r="V6" s="10"/>
+    </row>
+    <row r="7" spans="1:35" s="11" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+      <c r="A7" s="8"/>
+      <c r="B7" s="21"/>
+      <c r="C7" s="22"/>
+      <c r="D7" s="22"/>
+      <c r="E7" s="23"/>
+      <c r="F7" s="8"/>
+      <c r="G7" s="9"/>
+      <c r="H7" s="9"/>
+      <c r="I7" s="9"/>
+      <c r="J7" s="8"/>
+      <c r="K7" s="8"/>
+      <c r="L7" s="8"/>
+      <c r="M7" s="12"/>
+      <c r="N7" s="9"/>
+      <c r="O7" s="9"/>
+      <c r="P7" s="9"/>
+      <c r="Q7" s="8"/>
+      <c r="R7" s="9"/>
+      <c r="S7" s="9"/>
+      <c r="T7" s="9"/>
+      <c r="U7" s="10"/>
+      <c r="V7" s="10"/>
+    </row>
+    <row r="8" spans="1:35" s="11" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+      <c r="A8" s="8"/>
+      <c r="B8" s="21"/>
+      <c r="C8" s="22"/>
+      <c r="D8" s="22"/>
+      <c r="E8" s="23"/>
+      <c r="F8" s="8"/>
+      <c r="G8" s="9"/>
+      <c r="H8" s="9"/>
+      <c r="I8" s="9"/>
+      <c r="J8" s="8"/>
+      <c r="K8" s="8"/>
+      <c r="L8" s="8"/>
+      <c r="M8" s="9"/>
+      <c r="N8" s="9"/>
+      <c r="O8" s="9"/>
+      <c r="P8" s="9"/>
+      <c r="Q8" s="8"/>
+      <c r="R8" s="9"/>
+      <c r="S8" s="9"/>
+      <c r="T8" s="9"/>
+      <c r="U8" s="10"/>
+      <c r="V8" s="10"/>
+    </row>
+    <row r="9" spans="1:35" s="11" customFormat="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="8"/>
+      <c r="B9" s="24"/>
+      <c r="C9" s="25"/>
+      <c r="D9" s="25"/>
+      <c r="E9" s="26"/>
+      <c r="F9" s="8"/>
+      <c r="G9" s="9"/>
+      <c r="H9" s="9"/>
+      <c r="I9" s="9"/>
+      <c r="J9" s="8"/>
+      <c r="K9" s="8"/>
+      <c r="L9" s="8"/>
+      <c r="M9" s="9"/>
+      <c r="N9" s="9"/>
+      <c r="O9" s="9"/>
+      <c r="P9" s="9"/>
+      <c r="Q9" s="8"/>
+      <c r="R9" s="9"/>
+      <c r="S9" s="9"/>
+      <c r="T9" s="9"/>
+      <c r="U9" s="10"/>
+      <c r="V9" s="10"/>
     </row>
     <row r="10" spans="1:35" customFormat="1" ht="19" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B10" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="C10" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="D10" s="1" t="s">
+      <c r="D10" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="E10" s="1" t="s">
+      <c r="E10" s="17" t="s">
         <v>22</v>
       </c>
       <c r="F10" s="1" t="s">
@@ -981,7 +1102,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="11" spans="1:35" s="8" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:35" s="7" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A11" s="4"/>
       <c r="B11" s="4"/>
       <c r="C11" s="4"/>
@@ -1002,23 +1123,23 @@
       <c r="R11" s="5"/>
       <c r="S11" s="5"/>
       <c r="T11" s="5"/>
-      <c r="U11" s="6"/>
-      <c r="V11" s="6"/>
-      <c r="W11" s="7"/>
-      <c r="X11" s="7"/>
-      <c r="Y11" s="7"/>
-      <c r="Z11" s="7"/>
-      <c r="AA11" s="7"/>
-      <c r="AB11" s="7"/>
-      <c r="AC11" s="7"/>
-      <c r="AD11" s="7"/>
-      <c r="AE11" s="7"/>
-      <c r="AF11" s="7"/>
-      <c r="AG11" s="7"/>
-      <c r="AH11" s="7"/>
-      <c r="AI11" s="7"/>
-    </row>
-    <row r="12" spans="1:35" s="8" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="U11" s="27"/>
+      <c r="V11" s="27"/>
+      <c r="W11" s="6"/>
+      <c r="X11" s="6"/>
+      <c r="Y11" s="6"/>
+      <c r="Z11" s="6"/>
+      <c r="AA11" s="6"/>
+      <c r="AB11" s="6"/>
+      <c r="AC11" s="6"/>
+      <c r="AD11" s="6"/>
+      <c r="AE11" s="6"/>
+      <c r="AF11" s="6"/>
+      <c r="AG11" s="6"/>
+      <c r="AH11" s="6"/>
+      <c r="AI11" s="6"/>
+    </row>
+    <row r="12" spans="1:35" s="7" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A12" s="4"/>
       <c r="B12" s="4"/>
       <c r="C12" s="4"/>
@@ -1039,23 +1160,23 @@
       <c r="R12" s="5"/>
       <c r="S12" s="5"/>
       <c r="T12" s="5"/>
-      <c r="U12" s="6"/>
-      <c r="V12" s="6"/>
-      <c r="W12" s="7"/>
-      <c r="X12" s="7"/>
-      <c r="Y12" s="7"/>
-      <c r="Z12" s="7"/>
-      <c r="AA12" s="7"/>
-      <c r="AB12" s="7"/>
-      <c r="AC12" s="7"/>
-      <c r="AD12" s="7"/>
-      <c r="AE12" s="7"/>
-      <c r="AF12" s="7"/>
-      <c r="AG12" s="7"/>
-      <c r="AH12" s="7"/>
-      <c r="AI12" s="7"/>
-    </row>
-    <row r="13" spans="1:35" s="8" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="U12" s="27"/>
+      <c r="V12" s="27"/>
+      <c r="W12" s="6"/>
+      <c r="X12" s="6"/>
+      <c r="Y12" s="6"/>
+      <c r="Z12" s="6"/>
+      <c r="AA12" s="6"/>
+      <c r="AB12" s="6"/>
+      <c r="AC12" s="6"/>
+      <c r="AD12" s="6"/>
+      <c r="AE12" s="6"/>
+      <c r="AF12" s="6"/>
+      <c r="AG12" s="6"/>
+      <c r="AH12" s="6"/>
+      <c r="AI12" s="6"/>
+    </row>
+    <row r="13" spans="1:35" s="7" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A13" s="4"/>
       <c r="B13" s="4"/>
       <c r="C13" s="4"/>
@@ -1076,23 +1197,23 @@
       <c r="R13" s="5"/>
       <c r="S13" s="5"/>
       <c r="T13" s="5"/>
-      <c r="U13" s="6"/>
-      <c r="V13" s="6"/>
-      <c r="W13" s="7"/>
-      <c r="X13" s="7"/>
-      <c r="Y13" s="7"/>
-      <c r="Z13" s="7"/>
-      <c r="AA13" s="7"/>
-      <c r="AB13" s="7"/>
-      <c r="AC13" s="7"/>
-      <c r="AD13" s="7"/>
-      <c r="AE13" s="7"/>
-      <c r="AF13" s="7"/>
-      <c r="AG13" s="7"/>
-      <c r="AH13" s="7"/>
-      <c r="AI13" s="7"/>
-    </row>
-    <row r="14" spans="1:35" s="8" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="U13" s="27"/>
+      <c r="V13" s="27"/>
+      <c r="W13" s="6"/>
+      <c r="X13" s="6"/>
+      <c r="Y13" s="6"/>
+      <c r="Z13" s="6"/>
+      <c r="AA13" s="6"/>
+      <c r="AB13" s="6"/>
+      <c r="AC13" s="6"/>
+      <c r="AD13" s="6"/>
+      <c r="AE13" s="6"/>
+      <c r="AF13" s="6"/>
+      <c r="AG13" s="6"/>
+      <c r="AH13" s="6"/>
+      <c r="AI13" s="6"/>
+    </row>
+    <row r="14" spans="1:35" s="7" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A14" s="4"/>
       <c r="B14" s="4"/>
       <c r="C14" s="4"/>
@@ -1113,23 +1234,23 @@
       <c r="R14" s="5"/>
       <c r="S14" s="5"/>
       <c r="T14" s="5"/>
-      <c r="U14" s="6"/>
-      <c r="V14" s="6"/>
-      <c r="W14" s="7"/>
-      <c r="X14" s="7"/>
-      <c r="Y14" s="7"/>
-      <c r="Z14" s="7"/>
-      <c r="AA14" s="7"/>
-      <c r="AB14" s="7"/>
-      <c r="AC14" s="7"/>
-      <c r="AD14" s="7"/>
-      <c r="AE14" s="7"/>
-      <c r="AF14" s="7"/>
-      <c r="AG14" s="7"/>
-      <c r="AH14" s="7"/>
-      <c r="AI14" s="7"/>
-    </row>
-    <row r="15" spans="1:35" s="8" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="U14" s="27"/>
+      <c r="V14" s="27"/>
+      <c r="W14" s="6"/>
+      <c r="X14" s="6"/>
+      <c r="Y14" s="6"/>
+      <c r="Z14" s="6"/>
+      <c r="AA14" s="6"/>
+      <c r="AB14" s="6"/>
+      <c r="AC14" s="6"/>
+      <c r="AD14" s="6"/>
+      <c r="AE14" s="6"/>
+      <c r="AF14" s="6"/>
+      <c r="AG14" s="6"/>
+      <c r="AH14" s="6"/>
+      <c r="AI14" s="6"/>
+    </row>
+    <row r="15" spans="1:35" s="7" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A15" s="4"/>
       <c r="B15" s="4"/>
       <c r="C15" s="4"/>
@@ -1150,26 +1271,25 @@
       <c r="R15" s="5"/>
       <c r="S15" s="5"/>
       <c r="T15" s="5"/>
-      <c r="U15" s="6"/>
-      <c r="V15" s="6"/>
-      <c r="W15" s="7"/>
-      <c r="X15" s="7"/>
-      <c r="Y15" s="7"/>
-      <c r="Z15" s="7"/>
-      <c r="AA15" s="7"/>
-      <c r="AB15" s="7"/>
-      <c r="AC15" s="7"/>
-      <c r="AD15" s="7"/>
-      <c r="AE15" s="7"/>
-      <c r="AF15" s="7"/>
-      <c r="AG15" s="7"/>
-      <c r="AH15" s="7"/>
-      <c r="AI15" s="7"/>
+      <c r="U15" s="27"/>
+      <c r="V15" s="27"/>
+      <c r="W15" s="6"/>
+      <c r="X15" s="6"/>
+      <c r="Y15" s="6"/>
+      <c r="Z15" s="6"/>
+      <c r="AA15" s="6"/>
+      <c r="AB15" s="6"/>
+      <c r="AC15" s="6"/>
+      <c r="AD15" s="6"/>
+      <c r="AE15" s="6"/>
+      <c r="AF15" s="6"/>
+      <c r="AG15" s="6"/>
+      <c r="AH15" s="6"/>
+      <c r="AI15" s="6"/>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A2:V2"/>
-    <mergeCell ref="A3:V3"/>
+  <mergeCells count="1">
+    <mergeCell ref="B1:E9"/>
   </mergeCells>
   <pageMargins left="0.70866141732283505" right="0.70866141732283505" top="0.74803149606299202" bottom="0.74803149606299202" header="0.31496062992126" footer="0.31496062992126"/>
   <pageSetup scale="28" fitToHeight="0" orientation="landscape" r:id="rId1"/>

</xml_diff>